<commit_message>
portfolio: cost of debt check note, drop unverified Paramount rating line
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YL7WQ5mcZJ4NppNnUaJjBS
</commit_message>
<xml_diff>
--- a/site_extra/portfolio/assets/Media_Credit_Comps.xlsx
+++ b/site_extra/portfolio/assets/Media_Credit_Comps.xlsx
@@ -478,7 +478,7 @@
     <t xml:space="preserve">Prices 46.53 to 62.90</t>
   </si>
   <si>
-    <t xml:space="preserve">Debtwire [1]. Now BB- at S&amp;P after the October 12 cut.</t>
+    <t xml:space="preserve">Debtwire [1]. Agency ratings on the legacy notes are not verified in this pass and are left out on purpose.</t>
   </si>
   <si>
     <t xml:space="preserve">Paramount Global 5 year CDS</t>
@@ -532,7 +532,7 @@
     <t xml:space="preserve">Ratings and levels not retrieved. $12 billion Morgan Stanley bridge and $1 billion term loan committed for Roku [2].</t>
   </si>
   <si>
-    <t xml:space="preserve">Three of the five have no sourced bond levels in this pass. On a terminal this sheet takes ten minutes to fill from YAS and the relative value screens. Without one I leave the cells empty rather than guess.</t>
+    <t xml:space="preserve">Three of the five have no sourced bond levels in this sheet. I have since checked the cost of debt inputs against where each name's paper trades on a Bloomberg Terminal. Those levels stay off this workbook and this site; the model inputs hold for Disney, Netflix and Fox, and Comcast's is the one the market has wider. Nothing here comes from a terminal.</t>
   </si>
   <si>
     <t xml:space="preserve">Sources</t>

</xml_diff>